<commit_message>
feat: implement correct heatmap values
</commit_message>
<xml_diff>
--- a/files/eGym-exercises-heatmap.xlsx
+++ b/files/eGym-exercises-heatmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Job\fitcode\fitcode\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0395A2E3-9F43-4E4A-BA5E-BF7C5C6E6978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE9F44EA-2271-45C3-867D-2BBFA3558F2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10441" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10501" uniqueCount="329">
   <si>
     <t>Half Squat - TB</t>
   </si>
@@ -980,9 +980,6 @@
     <t>erector_spinae_thoracis</t>
   </si>
   <si>
-    <t>erector_spinae_thoracis_2</t>
-  </si>
-  <si>
     <t>gastrocnemius-r_2</t>
   </si>
   <si>
@@ -1011,6 +1008,18 @@
   </si>
   <si>
     <t>wrist_extensors-l_2</t>
+  </si>
+  <si>
+    <t>extrenal_oblique-r_2</t>
+  </si>
+  <si>
+    <t>extrenal_oblique-l_2</t>
+  </si>
+  <si>
+    <t>gastrocnemius_front-r</t>
+  </si>
+  <si>
+    <t>gastrocnemius_front-l</t>
   </si>
 </sst>
 </file>
@@ -1436,7 +1445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH176"/>
+  <dimension ref="A1:BH177"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.88671875" style="2" customWidth="1"/>
@@ -5698,7 +5707,7 @@
     </row>
     <row r="26" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B26" t="s">
         <v>195</v>
@@ -5880,7 +5889,7 @@
     </row>
     <row r="27" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B27" t="s">
         <v>195</v>
@@ -19166,7 +19175,7 @@
     </row>
     <row r="100" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
-        <v>121</v>
+        <v>327</v>
       </c>
       <c r="B100" t="s">
         <v>192</v>
@@ -19348,7 +19357,7 @@
     </row>
     <row r="101" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
-        <v>122</v>
+        <v>328</v>
       </c>
       <c r="B101" t="s">
         <v>192</v>
@@ -20076,16 +20085,16 @@
     </row>
     <row r="105" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
-        <v>315</v>
+        <v>125</v>
       </c>
       <c r="B105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="C105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="D105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="E105" t="s">
         <v>176</v>
@@ -20094,127 +20103,127 @@
         <v>176</v>
       </c>
       <c r="G105" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="H105" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="I105" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J105" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="K105" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="L105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="M105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="N105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="O105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="P105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="Q105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="R105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="S105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="T105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="U105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="V105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="W105" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="X105" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="Y105" t="s">
+        <v>182</v>
+      </c>
+      <c r="Z105" t="s">
+        <v>182</v>
+      </c>
+      <c r="AA105" t="s">
+        <v>176</v>
+      </c>
+      <c r="AB105" t="s">
+        <v>182</v>
+      </c>
+      <c r="AC105" t="s">
+        <v>176</v>
+      </c>
+      <c r="AD105" t="s">
+        <v>175</v>
+      </c>
+      <c r="AE105" t="s">
+        <v>175</v>
+      </c>
+      <c r="AF105" t="s">
+        <v>175</v>
+      </c>
+      <c r="AG105" t="s">
+        <v>175</v>
+      </c>
+      <c r="AH105" t="s">
+        <v>182</v>
+      </c>
+      <c r="AI105" t="s">
         <v>183</v>
       </c>
-      <c r="Z105" t="s">
-        <v>197</v>
-      </c>
-      <c r="AA105" t="s">
-        <v>182</v>
-      </c>
-      <c r="AB105" t="s">
-        <v>197</v>
-      </c>
-      <c r="AC105" t="s">
-        <v>189</v>
-      </c>
-      <c r="AD105" t="s">
-        <v>176</v>
-      </c>
-      <c r="AE105" t="s">
-        <v>175</v>
-      </c>
-      <c r="AF105" t="s">
-        <v>175</v>
-      </c>
-      <c r="AG105" t="s">
-        <v>176</v>
-      </c>
-      <c r="AH105" t="s">
-        <v>195</v>
-      </c>
-      <c r="AI105" t="s">
-        <v>175</v>
-      </c>
       <c r="AJ105" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="AK105" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AL105" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="AM105" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="AN105" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AO105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="AP105" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="AQ105" t="s">
         <v>176</v>
       </c>
       <c r="AR105" t="s">
-        <v>195</v>
+        <v>233</v>
       </c>
       <c r="AS105" t="s">
-        <v>224</v>
+        <v>188</v>
       </c>
       <c r="AT105" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="AU105" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AV105" t="s">
         <v>176</v>
@@ -20223,42 +20232,42 @@
         <v>176</v>
       </c>
       <c r="AX105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="AY105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="AZ105" t="s">
         <v>224</v>
       </c>
       <c r="BA105" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="BB105" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="BC105" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="BD105" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="BE105" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="BF105" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="BG105" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="BH105" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
     </row>
     <row r="106" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B106" t="s">
         <v>175</v>
@@ -20440,7 +20449,7 @@
     </row>
     <row r="107" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B107" t="s">
         <v>175</v>
@@ -20569,7 +20578,7 @@
         <v>176</v>
       </c>
       <c r="AR107" t="s">
-        <v>233</v>
+        <v>255</v>
       </c>
       <c r="AS107" t="s">
         <v>188</v>
@@ -20622,7 +20631,7 @@
     </row>
     <row r="108" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B108" t="s">
         <v>175</v>
@@ -20804,16 +20813,16 @@
     </row>
     <row r="109" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
-        <v>128</v>
+        <v>312</v>
       </c>
       <c r="B109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E109" t="s">
         <v>176</v>
@@ -20828,46 +20837,46 @@
         <v>176</v>
       </c>
       <c r="I109" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J109" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K109" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="L109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="M109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="N109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="O109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="R109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="S109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W109" t="s">
         <v>180</v>
@@ -20891,16 +20900,16 @@
         <v>176</v>
       </c>
       <c r="AD109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AE109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AF109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AG109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AH109" t="s">
         <v>182</v>
@@ -20924,7 +20933,7 @@
         <v>186</v>
       </c>
       <c r="AO109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AP109" t="s">
         <v>187</v>
@@ -20951,10 +20960,10 @@
         <v>176</v>
       </c>
       <c r="AX109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AY109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AZ109" t="s">
         <v>224</v>
@@ -20981,12 +20990,12 @@
         <v>176</v>
       </c>
       <c r="BH109" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="110" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B110" t="s">
         <v>176</v>
@@ -21168,16 +21177,16 @@
     </row>
     <row r="111" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
-        <v>313</v>
+        <v>129</v>
       </c>
       <c r="B111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E111" t="s">
         <v>176</v>
@@ -21186,52 +21195,52 @@
         <v>176</v>
       </c>
       <c r="G111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I111" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J111" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="K111" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="L111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="M111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="N111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="O111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="P111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Q111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="S111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="V111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="W111" t="s">
         <v>180</v>
@@ -21240,40 +21249,40 @@
         <v>176</v>
       </c>
       <c r="Y111" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="Z111" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AA111" t="s">
         <v>176</v>
       </c>
       <c r="AB111" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AC111" t="s">
         <v>176</v>
       </c>
       <c r="AD111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AE111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AF111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AG111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AH111" t="s">
         <v>182</v>
       </c>
       <c r="AI111" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="AJ111" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="AK111" t="s">
         <v>176</v>
@@ -21288,7 +21297,7 @@
         <v>186</v>
       </c>
       <c r="AO111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AP111" t="s">
         <v>187</v>
@@ -21297,10 +21306,10 @@
         <v>176</v>
       </c>
       <c r="AR111" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="AS111" t="s">
-        <v>188</v>
+        <v>217</v>
       </c>
       <c r="AT111" t="s">
         <v>176</v>
@@ -21315,42 +21324,42 @@
         <v>176</v>
       </c>
       <c r="AX111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AY111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AZ111" t="s">
         <v>224</v>
       </c>
       <c r="BA111" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="BB111" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="BC111" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="BD111" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="BE111" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="BF111" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="BG111" t="s">
         <v>176</v>
       </c>
       <c r="BH111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="112" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B112" t="s">
         <v>175</v>
@@ -21532,7 +21541,7 @@
     </row>
     <row r="113" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B113" t="s">
         <v>175</v>
@@ -21714,7 +21723,7 @@
     </row>
     <row r="114" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B114" t="s">
         <v>175</v>
@@ -21896,7 +21905,7 @@
     </row>
     <row r="115" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B115" t="s">
         <v>175</v>
@@ -21908,25 +21917,25 @@
         <v>175</v>
       </c>
       <c r="E115" t="s">
-        <v>176</v>
+        <v>262</v>
       </c>
       <c r="F115" t="s">
         <v>176</v>
       </c>
       <c r="G115" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H115" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I115" t="s">
-        <v>177</v>
+        <v>218</v>
       </c>
       <c r="J115" t="s">
         <v>178</v>
       </c>
       <c r="K115" t="s">
-        <v>179</v>
+        <v>211</v>
       </c>
       <c r="L115" t="s">
         <v>175</v>
@@ -21962,7 +21971,7 @@
         <v>175</v>
       </c>
       <c r="W115" t="s">
-        <v>180</v>
+        <v>218</v>
       </c>
       <c r="X115" t="s">
         <v>176</v>
@@ -21983,52 +21992,52 @@
         <v>176</v>
       </c>
       <c r="AD115" t="s">
-        <v>175</v>
+        <v>213</v>
       </c>
       <c r="AE115" t="s">
-        <v>175</v>
+        <v>213</v>
       </c>
       <c r="AF115" t="s">
-        <v>175</v>
+        <v>213</v>
       </c>
       <c r="AG115" t="s">
-        <v>175</v>
+        <v>213</v>
       </c>
       <c r="AH115" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="AI115" t="s">
-        <v>175</v>
+        <v>214</v>
       </c>
       <c r="AJ115" t="s">
-        <v>175</v>
+        <v>214</v>
       </c>
       <c r="AK115" t="s">
         <v>176</v>
       </c>
       <c r="AL115" t="s">
-        <v>184</v>
+        <v>213</v>
       </c>
       <c r="AM115" t="s">
         <v>185</v>
       </c>
       <c r="AN115" t="s">
-        <v>186</v>
+        <v>213</v>
       </c>
       <c r="AO115" t="s">
         <v>175</v>
       </c>
       <c r="AP115" t="s">
-        <v>187</v>
+        <v>263</v>
       </c>
       <c r="AQ115" t="s">
         <v>176</v>
       </c>
       <c r="AR115" t="s">
-        <v>261</v>
+        <v>175</v>
       </c>
       <c r="AS115" t="s">
-        <v>217</v>
+        <v>264</v>
       </c>
       <c r="AT115" t="s">
         <v>176</v>
@@ -22049,7 +22058,7 @@
         <v>175</v>
       </c>
       <c r="AZ115" t="s">
-        <v>224</v>
+        <v>189</v>
       </c>
       <c r="BA115" t="s">
         <v>176</v>
@@ -22078,7 +22087,7 @@
     </row>
     <row r="116" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B116" t="s">
         <v>175</v>
@@ -22260,7 +22269,7 @@
     </row>
     <row r="117" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B117" t="s">
         <v>175</v>
@@ -22442,7 +22451,7 @@
     </row>
     <row r="118" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B118" t="s">
         <v>175</v>
@@ -22624,7 +22633,7 @@
     </row>
     <row r="119" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
-        <v>136</v>
+        <v>311</v>
       </c>
       <c r="B119" t="s">
         <v>175</v>
@@ -22753,10 +22762,10 @@
         <v>176</v>
       </c>
       <c r="AR119" t="s">
-        <v>175</v>
+        <v>255</v>
       </c>
       <c r="AS119" t="s">
-        <v>264</v>
+        <v>216</v>
       </c>
       <c r="AT119" t="s">
         <v>176</v>
@@ -22806,7 +22815,7 @@
     </row>
     <row r="120" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
-        <v>311</v>
+        <v>137</v>
       </c>
       <c r="B120" t="s">
         <v>175</v>
@@ -22988,145 +22997,145 @@
     </row>
     <row r="121" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E121" t="s">
-        <v>262</v>
+        <v>176</v>
       </c>
       <c r="F121" t="s">
         <v>176</v>
       </c>
       <c r="G121" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H121" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I121" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J121" t="s">
-        <v>178</v>
+        <v>219</v>
       </c>
       <c r="K121" t="s">
-        <v>211</v>
+        <v>176</v>
       </c>
       <c r="L121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="M121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="N121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="O121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="R121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="S121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W121" t="s">
-        <v>218</v>
+        <v>176</v>
       </c>
       <c r="X121" t="s">
         <v>176</v>
       </c>
       <c r="Y121" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="Z121" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AA121" t="s">
         <v>176</v>
       </c>
       <c r="AB121" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AC121" t="s">
         <v>176</v>
       </c>
       <c r="AD121" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="AE121" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="AF121" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="AG121" t="s">
-        <v>213</v>
+        <v>181</v>
       </c>
       <c r="AH121" t="s">
         <v>189</v>
       </c>
       <c r="AI121" t="s">
-        <v>214</v>
+        <v>176</v>
       </c>
       <c r="AJ121" t="s">
-        <v>214</v>
+        <v>176</v>
       </c>
       <c r="AK121" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AL121" t="s">
-        <v>213</v>
+        <v>265</v>
       </c>
       <c r="AM121" t="s">
-        <v>185</v>
+        <v>266</v>
       </c>
       <c r="AN121" t="s">
         <v>213</v>
       </c>
       <c r="AO121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AP121" t="s">
-        <v>263</v>
+        <v>239</v>
       </c>
       <c r="AQ121" t="s">
         <v>176</v>
       </c>
       <c r="AR121" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="AS121" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AT121" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AU121" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AV121" t="s">
         <v>176</v>
@@ -23135,42 +23144,42 @@
         <v>176</v>
       </c>
       <c r="AX121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AY121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AZ121" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="BA121" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BB121" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BC121" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BD121" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BE121" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BF121" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BG121" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="BH121" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="122" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B122" t="s">
         <v>176</v>
@@ -23352,145 +23361,145 @@
     </row>
     <row r="123" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E123" t="s">
-        <v>176</v>
+        <v>262</v>
       </c>
       <c r="F123" t="s">
         <v>176</v>
       </c>
       <c r="G123" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H123" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I123" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J123" t="s">
-        <v>219</v>
+        <v>178</v>
       </c>
       <c r="K123" t="s">
-        <v>176</v>
+        <v>211</v>
       </c>
       <c r="L123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="M123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="N123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="O123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="P123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Q123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="S123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="V123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="W123" t="s">
-        <v>176</v>
+        <v>268</v>
       </c>
       <c r="X123" t="s">
         <v>176</v>
       </c>
       <c r="Y123" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="Z123" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AA123" t="s">
         <v>176</v>
       </c>
       <c r="AB123" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AC123" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="AD123" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="AE123" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="AF123" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="AG123" t="s">
-        <v>181</v>
+        <v>220</v>
       </c>
       <c r="AH123" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="AI123" t="s">
-        <v>176</v>
+        <v>221</v>
       </c>
       <c r="AJ123" t="s">
-        <v>176</v>
+        <v>221</v>
       </c>
       <c r="AK123" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AL123" t="s">
-        <v>265</v>
+        <v>214</v>
       </c>
       <c r="AM123" t="s">
-        <v>266</v>
+        <v>188</v>
       </c>
       <c r="AN123" t="s">
         <v>213</v>
       </c>
       <c r="AO123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AP123" t="s">
-        <v>239</v>
+        <v>222</v>
       </c>
       <c r="AQ123" t="s">
         <v>176</v>
       </c>
       <c r="AR123" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="AS123" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="AT123" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="AU123" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AV123" t="s">
         <v>176</v>
@@ -23499,42 +23508,42 @@
         <v>176</v>
       </c>
       <c r="AX123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AY123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AZ123" t="s">
-        <v>208</v>
+        <v>189</v>
       </c>
       <c r="BA123" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="BB123" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="BC123" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="BD123" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="BE123" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="BF123" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="BG123" t="s">
-        <v>189</v>
+        <v>224</v>
       </c>
       <c r="BH123" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="124" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B124" t="s">
         <v>175</v>
@@ -23716,7 +23725,7 @@
     </row>
     <row r="125" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
-        <v>141</v>
+        <v>304</v>
       </c>
       <c r="B125" t="s">
         <v>175</v>
@@ -23740,7 +23749,7 @@
         <v>176</v>
       </c>
       <c r="I125" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J125" t="s">
         <v>178</v>
@@ -23898,7 +23907,7 @@
     </row>
     <row r="126" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B126" t="s">
         <v>175</v>
@@ -24080,79 +24089,79 @@
     </row>
     <row r="127" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
-        <v>305</v>
+        <v>86</v>
       </c>
       <c r="B127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E127" t="s">
-        <v>262</v>
+        <v>176</v>
       </c>
       <c r="F127" t="s">
         <v>176</v>
       </c>
       <c r="G127" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="H127" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="I127" t="s">
         <v>219</v>
       </c>
       <c r="J127" t="s">
-        <v>178</v>
+        <v>218</v>
       </c>
       <c r="K127" t="s">
-        <v>211</v>
+        <v>176</v>
       </c>
       <c r="L127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="M127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="N127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="O127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="R127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="S127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="T127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W127" t="s">
-        <v>268</v>
+        <v>222</v>
       </c>
       <c r="X127" t="s">
         <v>176</v>
       </c>
       <c r="Y127" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="Z127" t="s">
         <v>176</v>
@@ -24167,25 +24176,25 @@
         <v>183</v>
       </c>
       <c r="AD127" t="s">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="AE127" t="s">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="AF127" t="s">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="AG127" t="s">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="AH127" t="s">
         <v>176</v>
       </c>
       <c r="AI127" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="AJ127" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="AK127" t="s">
         <v>176</v>
@@ -24194,13 +24203,13 @@
         <v>214</v>
       </c>
       <c r="AM127" t="s">
-        <v>188</v>
+        <v>217</v>
       </c>
       <c r="AN127" t="s">
-        <v>213</v>
+        <v>178</v>
       </c>
       <c r="AO127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AP127" t="s">
         <v>222</v>
@@ -24212,7 +24221,7 @@
         <v>255</v>
       </c>
       <c r="AS127" t="s">
-        <v>213</v>
+        <v>182</v>
       </c>
       <c r="AT127" t="s">
         <v>176</v>
@@ -24227,42 +24236,42 @@
         <v>176</v>
       </c>
       <c r="AX127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AY127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AZ127" t="s">
         <v>189</v>
       </c>
       <c r="BA127" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="BB127" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="BC127" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="BD127" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="BE127" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="BF127" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="BG127" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="BH127" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="128" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B128" t="s">
         <v>176</v>
@@ -24444,7 +24453,7 @@
     </row>
     <row r="129" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
-        <v>87</v>
+        <v>142</v>
       </c>
       <c r="B129" t="s">
         <v>176</v>
@@ -24468,10 +24477,10 @@
         <v>193</v>
       </c>
       <c r="I129" t="s">
-        <v>219</v>
+        <v>176</v>
       </c>
       <c r="J129" t="s">
-        <v>218</v>
+        <v>176</v>
       </c>
       <c r="K129" t="s">
         <v>176</v>
@@ -24626,7 +24635,7 @@
     </row>
     <row r="130" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B130" t="s">
         <v>176</v>
@@ -24808,7 +24817,7 @@
     </row>
     <row r="131" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B131" t="s">
         <v>176</v>
@@ -24990,7 +24999,7 @@
     </row>
     <row r="132" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B132" t="s">
         <v>176</v>
@@ -25172,7 +25181,7 @@
     </row>
     <row r="133" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B133" t="s">
         <v>176</v>
@@ -25184,16 +25193,16 @@
         <v>176</v>
       </c>
       <c r="E133" t="s">
-        <v>176</v>
+        <v>218</v>
       </c>
       <c r="F133" t="s">
         <v>176</v>
       </c>
       <c r="G133" t="s">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="H133" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="I133" t="s">
         <v>176</v>
@@ -25238,7 +25247,7 @@
         <v>176</v>
       </c>
       <c r="W133" t="s">
-        <v>222</v>
+        <v>176</v>
       </c>
       <c r="X133" t="s">
         <v>176</v>
@@ -25256,52 +25265,52 @@
         <v>176</v>
       </c>
       <c r="AC133" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="AD133" t="s">
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="AE133" t="s">
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="AF133" t="s">
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="AG133" t="s">
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="AH133" t="s">
         <v>176</v>
       </c>
       <c r="AI133" t="s">
-        <v>226</v>
+        <v>189</v>
       </c>
       <c r="AJ133" t="s">
-        <v>226</v>
+        <v>189</v>
       </c>
       <c r="AK133" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AL133" t="s">
-        <v>214</v>
+        <v>175</v>
       </c>
       <c r="AM133" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="AN133" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="AO133" t="s">
         <v>176</v>
       </c>
       <c r="AP133" t="s">
-        <v>222</v>
+        <v>182</v>
       </c>
       <c r="AQ133" t="s">
         <v>176</v>
       </c>
       <c r="AR133" t="s">
-        <v>255</v>
+        <v>189</v>
       </c>
       <c r="AS133" t="s">
         <v>182</v>
@@ -25325,7 +25334,7 @@
         <v>176</v>
       </c>
       <c r="AZ133" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="BA133" t="s">
         <v>176</v>
@@ -25346,7 +25355,7 @@
         <v>176</v>
       </c>
       <c r="BG133" t="s">
-        <v>227</v>
+        <v>189</v>
       </c>
       <c r="BH133" t="s">
         <v>176</v>
@@ -25354,7 +25363,7 @@
     </row>
     <row r="134" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B134" t="s">
         <v>176</v>
@@ -25536,7 +25545,7 @@
     </row>
     <row r="135" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
-        <v>147</v>
+        <v>323</v>
       </c>
       <c r="B135" t="s">
         <v>176</v>
@@ -25900,7 +25909,7 @@
     </row>
     <row r="137" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
-        <v>325</v>
+        <v>148</v>
       </c>
       <c r="B137" t="s">
         <v>176</v>
@@ -26053,7 +26062,7 @@
         <v>176</v>
       </c>
       <c r="AZ137" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="BA137" t="s">
         <v>176</v>
@@ -26074,7 +26083,7 @@
         <v>176</v>
       </c>
       <c r="BG137" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="BH137" t="s">
         <v>176</v>
@@ -26082,7 +26091,7 @@
     </row>
     <row r="138" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B138" t="s">
         <v>176</v>
@@ -26264,7 +26273,7 @@
     </row>
     <row r="139" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B139" t="s">
         <v>176</v>
@@ -26276,16 +26285,16 @@
         <v>176</v>
       </c>
       <c r="E139" t="s">
-        <v>218</v>
+        <v>176</v>
       </c>
       <c r="F139" t="s">
         <v>176</v>
       </c>
       <c r="G139" t="s">
-        <v>269</v>
+        <v>176</v>
       </c>
       <c r="H139" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I139" t="s">
         <v>176</v>
@@ -26351,37 +26360,37 @@
         <v>176</v>
       </c>
       <c r="AD139" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AE139" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AF139" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AG139" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AH139" t="s">
         <v>176</v>
       </c>
       <c r="AI139" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="AJ139" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="AK139" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AL139" t="s">
         <v>175</v>
       </c>
       <c r="AM139" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="AN139" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AO139" t="s">
         <v>176</v>
@@ -26396,7 +26405,7 @@
         <v>189</v>
       </c>
       <c r="AS139" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AT139" t="s">
         <v>176</v>
@@ -26446,7 +26455,7 @@
     </row>
     <row r="140" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B140" t="s">
         <v>176</v>
@@ -26518,7 +26527,7 @@
         <v>176</v>
       </c>
       <c r="Y140" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="Z140" t="s">
         <v>176</v>
@@ -26569,16 +26578,16 @@
         <v>176</v>
       </c>
       <c r="AP140" t="s">
-        <v>182</v>
+        <v>270</v>
       </c>
       <c r="AQ140" t="s">
         <v>176</v>
       </c>
       <c r="AR140" t="s">
-        <v>189</v>
+        <v>255</v>
       </c>
       <c r="AS140" t="s">
-        <v>176</v>
+        <v>217</v>
       </c>
       <c r="AT140" t="s">
         <v>176</v>
@@ -26599,7 +26608,7 @@
         <v>176</v>
       </c>
       <c r="AZ140" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="BA140" t="s">
         <v>176</v>
@@ -26628,7 +26637,7 @@
     </row>
     <row r="141" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B141" t="s">
         <v>176</v>
@@ -26810,22 +26819,22 @@
     </row>
     <row r="142" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="C142" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="D142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="E142" t="s">
         <v>176</v>
       </c>
       <c r="F142" t="s">
-        <v>176</v>
+        <v>271</v>
       </c>
       <c r="G142" t="s">
         <v>176</v>
@@ -26834,165 +26843,165 @@
         <v>176</v>
       </c>
       <c r="I142" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="J142" t="s">
-        <v>176</v>
+        <v>216</v>
       </c>
       <c r="K142" t="s">
         <v>176</v>
       </c>
       <c r="L142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="M142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="N142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="O142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="P142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="Q142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="R142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="S142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="T142" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="U142" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="V142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="W142" t="s">
-        <v>176</v>
+        <v>222</v>
       </c>
       <c r="X142" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="Y142" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="Z142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="AA142" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="AB142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="AC142" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="AD142" t="s">
         <v>176</v>
       </c>
       <c r="AE142" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AF142" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AG142" t="s">
         <v>176</v>
       </c>
       <c r="AH142" t="s">
-        <v>176</v>
+        <v>241</v>
       </c>
       <c r="AI142" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AJ142" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AK142" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="AL142" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AM142" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AN142" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="AO142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="AP142" t="s">
-        <v>270</v>
+        <v>189</v>
       </c>
       <c r="AQ142" t="s">
-        <v>176</v>
+        <v>272</v>
       </c>
       <c r="AR142" t="s">
+        <v>189</v>
+      </c>
+      <c r="AS142" t="s">
+        <v>182</v>
+      </c>
+      <c r="AT142" t="s">
+        <v>273</v>
+      </c>
+      <c r="AU142" t="s">
+        <v>195</v>
+      </c>
+      <c r="AV142" t="s">
+        <v>244</v>
+      </c>
+      <c r="AW142" t="s">
+        <v>244</v>
+      </c>
+      <c r="AX142" t="s">
+        <v>244</v>
+      </c>
+      <c r="AY142" t="s">
+        <v>244</v>
+      </c>
+      <c r="AZ142" t="s">
         <v>255</v>
       </c>
-      <c r="AS142" t="s">
-        <v>217</v>
-      </c>
-      <c r="AT142" t="s">
-        <v>176</v>
-      </c>
-      <c r="AU142" t="s">
-        <v>176</v>
-      </c>
-      <c r="AV142" t="s">
-        <v>176</v>
-      </c>
-      <c r="AW142" t="s">
-        <v>176</v>
-      </c>
-      <c r="AX142" t="s">
-        <v>176</v>
-      </c>
-      <c r="AY142" t="s">
-        <v>176</v>
-      </c>
-      <c r="AZ142" t="s">
-        <v>189</v>
-      </c>
       <c r="BA142" t="s">
-        <v>176</v>
+        <v>241</v>
       </c>
       <c r="BB142" t="s">
-        <v>176</v>
+        <v>241</v>
       </c>
       <c r="BC142" t="s">
-        <v>176</v>
+        <v>241</v>
       </c>
       <c r="BD142" t="s">
-        <v>176</v>
+        <v>241</v>
       </c>
       <c r="BE142" t="s">
-        <v>176</v>
+        <v>241</v>
       </c>
       <c r="BF142" t="s">
-        <v>176</v>
+        <v>241</v>
       </c>
       <c r="BG142" t="s">
         <v>176</v>
       </c>
       <c r="BH142" t="s">
-        <v>176</v>
+        <v>244</v>
       </c>
     </row>
     <row r="143" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B143" t="s">
         <v>244</v>
@@ -27174,7 +27183,7 @@
     </row>
     <row r="144" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B144" t="s">
         <v>244</v>
@@ -27356,7 +27365,7 @@
     </row>
     <row r="145" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B145" t="s">
         <v>244</v>
@@ -27538,7 +27547,7 @@
     </row>
     <row r="146" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B146" t="s">
         <v>244</v>
@@ -27720,7 +27729,7 @@
     </row>
     <row r="147" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B147" t="s">
         <v>244</v>
@@ -27902,94 +27911,94 @@
     </row>
     <row r="148" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
-        <v>158</v>
+        <v>74</v>
       </c>
       <c r="B148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="C148" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="E148" t="s">
         <v>176</v>
       </c>
       <c r="F148" t="s">
-        <v>271</v>
+        <v>189</v>
       </c>
       <c r="G148" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="H148" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="I148" t="s">
-        <v>180</v>
+        <v>203</v>
       </c>
       <c r="J148" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="K148" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="L148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="M148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="N148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="O148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="P148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="Q148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="R148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="S148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="T148" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="U148" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="V148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="W148" t="s">
-        <v>222</v>
+        <v>189</v>
       </c>
       <c r="X148" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="Y148" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="Z148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="AA148" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="AB148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="AC148" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="AD148" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AE148" t="s">
         <v>175</v>
@@ -27998,93 +28007,93 @@
         <v>175</v>
       </c>
       <c r="AG148" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AH148" t="s">
-        <v>241</v>
+        <v>195</v>
       </c>
       <c r="AI148" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="AJ148" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="AK148" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="AL148" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="AM148" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="AN148" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="AO148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="AP148" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="AQ148" t="s">
-        <v>272</v>
+        <v>175</v>
       </c>
       <c r="AR148" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="AS148" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="AT148" t="s">
-        <v>273</v>
+        <v>189</v>
       </c>
       <c r="AU148" t="s">
         <v>195</v>
       </c>
       <c r="AV148" t="s">
-        <v>244</v>
+        <v>201</v>
       </c>
       <c r="AW148" t="s">
-        <v>244</v>
+        <v>201</v>
       </c>
       <c r="AX148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="AY148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="AZ148" t="s">
-        <v>255</v>
+        <v>202</v>
       </c>
       <c r="BA148" t="s">
-        <v>241</v>
+        <v>195</v>
       </c>
       <c r="BB148" t="s">
-        <v>241</v>
+        <v>195</v>
       </c>
       <c r="BC148" t="s">
-        <v>241</v>
+        <v>195</v>
       </c>
       <c r="BD148" t="s">
-        <v>241</v>
+        <v>195</v>
       </c>
       <c r="BE148" t="s">
-        <v>241</v>
+        <v>195</v>
       </c>
       <c r="BF148" t="s">
-        <v>241</v>
+        <v>195</v>
       </c>
       <c r="BG148" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="BH148" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
     </row>
     <row r="149" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B149" t="s">
         <v>195</v>
@@ -28266,7 +28275,7 @@
     </row>
     <row r="150" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
-        <v>75</v>
+        <v>159</v>
       </c>
       <c r="B150" t="s">
         <v>195</v>
@@ -28448,7 +28457,7 @@
     </row>
     <row r="151" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B151" t="s">
         <v>195</v>
@@ -28630,7 +28639,7 @@
     </row>
     <row r="152" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
-        <v>160</v>
+        <v>325</v>
       </c>
       <c r="B152" t="s">
         <v>195</v>
@@ -28812,189 +28821,189 @@
     </row>
     <row r="153" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
-        <v>161</v>
+        <v>326</v>
       </c>
       <c r="B153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="C153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="D153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="E153" t="s">
         <v>176</v>
       </c>
       <c r="F153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="G153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="H153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="I153" t="s">
-        <v>176</v>
+        <v>203</v>
       </c>
       <c r="J153" t="s">
-        <v>176</v>
+        <v>199</v>
       </c>
       <c r="K153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="L153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="M153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="N153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="O153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="P153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="Q153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="R153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="S153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="T153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="U153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="V153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="W153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="X153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="Y153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="Z153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AA153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AB153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AC153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AD153" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AE153" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AF153" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AG153" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AH153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AI153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="AJ153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="AK153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AL153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="AM153" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="AN153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="AO153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AP153" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="AQ153" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AR153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AS153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="AT153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="AU153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AV153" t="s">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="AW153" t="s">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="AX153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AY153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="AZ153" t="s">
-        <v>176</v>
+        <v>202</v>
       </c>
       <c r="BA153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BB153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BC153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BD153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BE153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BF153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BG153" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="BH153" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
     </row>
     <row r="154" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B154" t="s">
         <v>176</v>
@@ -29176,16 +29185,16 @@
     </row>
     <row r="155" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
-        <v>117</v>
+        <v>162</v>
       </c>
       <c r="B155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="C155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="D155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="E155" t="s">
         <v>176</v>
@@ -29209,37 +29218,37 @@
         <v>176</v>
       </c>
       <c r="L155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="M155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="N155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="O155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="P155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="Q155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="R155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="S155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="T155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="U155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="V155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="W155" t="s">
         <v>176</v>
@@ -29275,7 +29284,7 @@
         <v>176</v>
       </c>
       <c r="AH155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="AI155" t="s">
         <v>176</v>
@@ -29290,25 +29299,25 @@
         <v>176</v>
       </c>
       <c r="AM155" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AN155" t="s">
-        <v>222</v>
+        <v>176</v>
       </c>
       <c r="AO155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="AP155" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="AQ155" t="s">
         <v>176</v>
       </c>
       <c r="AR155" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AS155" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AT155" t="s">
         <v>176</v>
@@ -29323,42 +29332,42 @@
         <v>176</v>
       </c>
       <c r="AX155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="AY155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="AZ155" t="s">
         <v>176</v>
       </c>
       <c r="BA155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="BB155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="BC155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="BD155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="BE155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="BF155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="BG155" t="s">
         <v>176</v>
       </c>
       <c r="BH155" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
     </row>
     <row r="156" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B156" t="s">
         <v>250</v>
@@ -29499,10 +29508,10 @@
         <v>176</v>
       </c>
       <c r="AV156" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="AW156" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="AX156" t="s">
         <v>250</v>
@@ -29540,16 +29549,16 @@
     </row>
     <row r="157" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
-        <v>163</v>
+        <v>118</v>
       </c>
       <c r="B157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="C157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="D157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="E157" t="s">
         <v>176</v>
@@ -29573,100 +29582,100 @@
         <v>176</v>
       </c>
       <c r="L157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="M157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="N157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="O157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="P157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="Q157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="R157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="S157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="T157" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="U157" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="V157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="W157" t="s">
-        <v>261</v>
+        <v>176</v>
       </c>
       <c r="X157" t="s">
-        <v>274</v>
+        <v>176</v>
       </c>
       <c r="Y157" t="s">
-        <v>193</v>
+        <v>176</v>
       </c>
       <c r="Z157" t="s">
-        <v>244</v>
+        <v>176</v>
       </c>
       <c r="AA157" t="s">
-        <v>274</v>
+        <v>176</v>
       </c>
       <c r="AB157" t="s">
-        <v>244</v>
+        <v>176</v>
       </c>
       <c r="AC157" t="s">
-        <v>193</v>
+        <v>176</v>
       </c>
       <c r="AD157" t="s">
         <v>176</v>
       </c>
       <c r="AE157" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AF157" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AG157" t="s">
         <v>176</v>
       </c>
       <c r="AH157" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="AI157" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AJ157" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AK157" t="s">
-        <v>244</v>
+        <v>176</v>
       </c>
       <c r="AL157" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AM157" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AN157" t="s">
         <v>222</v>
       </c>
       <c r="AO157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="AP157" t="s">
         <v>182</v>
       </c>
       <c r="AQ157" t="s">
-        <v>237</v>
+        <v>176</v>
       </c>
       <c r="AR157" t="s">
         <v>182</v>
@@ -29675,10 +29684,10 @@
         <v>182</v>
       </c>
       <c r="AT157" t="s">
-        <v>273</v>
+        <v>176</v>
       </c>
       <c r="AU157" t="s">
-        <v>250</v>
+        <v>176</v>
       </c>
       <c r="AV157" t="s">
         <v>242</v>
@@ -29687,42 +29696,42 @@
         <v>242</v>
       </c>
       <c r="AX157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="AY157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="AZ157" t="s">
-        <v>207</v>
+        <v>176</v>
       </c>
       <c r="BA157" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="BB157" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="BC157" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="BD157" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="BE157" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="BF157" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="BG157" t="s">
         <v>176</v>
       </c>
       <c r="BH157" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
     </row>
     <row r="158" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B158" t="s">
         <v>256</v>
@@ -29904,7 +29913,7 @@
     </row>
     <row r="159" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B159" t="s">
         <v>256</v>
@@ -30086,7 +30095,7 @@
     </row>
     <row r="160" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B160" t="s">
         <v>256</v>
@@ -30268,7 +30277,7 @@
     </row>
     <row r="161" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B161" t="s">
         <v>256</v>
@@ -30337,7 +30346,7 @@
         <v>261</v>
       </c>
       <c r="X161" t="s">
-        <v>176</v>
+        <v>274</v>
       </c>
       <c r="Y161" t="s">
         <v>193</v>
@@ -30346,7 +30355,7 @@
         <v>244</v>
       </c>
       <c r="AA161" t="s">
-        <v>176</v>
+        <v>274</v>
       </c>
       <c r="AB161" t="s">
         <v>244</v>
@@ -30379,7 +30388,7 @@
         <v>244</v>
       </c>
       <c r="AL161" t="s">
-        <v>275</v>
+        <v>175</v>
       </c>
       <c r="AM161" t="s">
         <v>175</v>
@@ -30391,10 +30400,10 @@
         <v>256</v>
       </c>
       <c r="AP161" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AQ161" t="s">
-        <v>176</v>
+        <v>237</v>
       </c>
       <c r="AR161" t="s">
         <v>182</v>
@@ -30442,7 +30451,7 @@
         <v>235</v>
       </c>
       <c r="BG161" t="s">
-        <v>232</v>
+        <v>176</v>
       </c>
       <c r="BH161" t="s">
         <v>256</v>
@@ -30450,7 +30459,7 @@
     </row>
     <row r="162" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B162" t="s">
         <v>256</v>
@@ -30632,7 +30641,7 @@
     </row>
     <row r="163" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B163" t="s">
         <v>256</v>
@@ -30814,7 +30823,7 @@
     </row>
     <row r="164" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B164" t="s">
         <v>256</v>
@@ -30996,22 +31005,22 @@
     </row>
     <row r="165" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
-        <v>121</v>
+        <v>170</v>
       </c>
       <c r="B165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="C165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="D165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="E165" t="s">
         <v>176</v>
       </c>
       <c r="F165" t="s">
-        <v>217</v>
+        <v>176</v>
       </c>
       <c r="G165" t="s">
         <v>176</v>
@@ -31029,58 +31038,58 @@
         <v>176</v>
       </c>
       <c r="L165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="M165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="N165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="O165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="P165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="Q165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="R165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="S165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="T165" t="s">
-        <v>192</v>
+        <v>235</v>
       </c>
       <c r="U165" t="s">
-        <v>192</v>
+        <v>235</v>
       </c>
       <c r="V165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="W165" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="X165" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="Y165" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="Z165" t="s">
-        <v>192</v>
+        <v>244</v>
       </c>
       <c r="AA165" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="AB165" t="s">
-        <v>192</v>
+        <v>244</v>
       </c>
       <c r="AC165" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="AD165" t="s">
         <v>176</v>
@@ -31095,7 +31104,7 @@
         <v>176</v>
       </c>
       <c r="AH165" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
       <c r="AI165" t="s">
         <v>175</v>
@@ -31104,10 +31113,10 @@
         <v>175</v>
       </c>
       <c r="AK165" t="s">
-        <v>192</v>
+        <v>244</v>
       </c>
       <c r="AL165" t="s">
-        <v>175</v>
+        <v>275</v>
       </c>
       <c r="AM165" t="s">
         <v>175</v>
@@ -31116,10 +31125,10 @@
         <v>222</v>
       </c>
       <c r="AO165" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="AP165" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="AQ165" t="s">
         <v>176</v>
@@ -31128,13 +31137,13 @@
         <v>182</v>
       </c>
       <c r="AS165" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AT165" t="s">
-        <v>241</v>
+        <v>273</v>
       </c>
       <c r="AU165" t="s">
-        <v>276</v>
+        <v>250</v>
       </c>
       <c r="AV165" t="s">
         <v>242</v>
@@ -31143,42 +31152,42 @@
         <v>242</v>
       </c>
       <c r="AX165" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="AY165" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="AZ165" t="s">
-        <v>176</v>
+        <v>207</v>
       </c>
       <c r="BA165" t="s">
+        <v>235</v>
+      </c>
+      <c r="BB165" t="s">
+        <v>235</v>
+      </c>
+      <c r="BC165" t="s">
+        <v>235</v>
+      </c>
+      <c r="BD165" t="s">
+        <v>235</v>
+      </c>
+      <c r="BE165" t="s">
+        <v>235</v>
+      </c>
+      <c r="BF165" t="s">
+        <v>235</v>
+      </c>
+      <c r="BG165" t="s">
+        <v>232</v>
+      </c>
+      <c r="BH165" t="s">
         <v>256</v>
-      </c>
-      <c r="BB165" t="s">
-        <v>256</v>
-      </c>
-      <c r="BC165" t="s">
-        <v>256</v>
-      </c>
-      <c r="BD165" t="s">
-        <v>256</v>
-      </c>
-      <c r="BE165" t="s">
-        <v>256</v>
-      </c>
-      <c r="BF165" t="s">
-        <v>256</v>
-      </c>
-      <c r="BG165" t="s">
-        <v>176</v>
-      </c>
-      <c r="BH165" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="166" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B166" t="s">
         <v>192</v>
@@ -31360,7 +31369,7 @@
     </row>
     <row r="167" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
-        <v>316</v>
+        <v>122</v>
       </c>
       <c r="B167" t="s">
         <v>192</v>
@@ -31542,7 +31551,7 @@
     </row>
     <row r="168" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B168" t="s">
         <v>192</v>
@@ -31724,22 +31733,22 @@
     </row>
     <row r="169" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
-        <v>171</v>
+        <v>316</v>
       </c>
       <c r="B169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="C169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="D169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="E169" t="s">
         <v>176</v>
       </c>
       <c r="F169" t="s">
-        <v>176</v>
+        <v>217</v>
       </c>
       <c r="G169" t="s">
         <v>176</v>
@@ -31757,58 +31766,58 @@
         <v>176</v>
       </c>
       <c r="L169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="M169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="N169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="O169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="P169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="Q169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="R169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="S169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="T169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="U169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="V169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="W169" t="s">
-        <v>176</v>
+        <v>255</v>
       </c>
       <c r="X169" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="Y169" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="Z169" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="AA169" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="AB169" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="AC169" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="AD169" t="s">
         <v>176</v>
@@ -31832,7 +31841,7 @@
         <v>175</v>
       </c>
       <c r="AK169" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="AL169" t="s">
         <v>175</v>
@@ -31841,13 +31850,13 @@
         <v>175</v>
       </c>
       <c r="AN169" t="s">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="AO169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
       <c r="AP169" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AQ169" t="s">
         <v>176</v>
@@ -31859,16 +31868,16 @@
         <v>176</v>
       </c>
       <c r="AT169" t="s">
-        <v>195</v>
+        <v>241</v>
       </c>
       <c r="AU169" t="s">
-        <v>176</v>
+        <v>276</v>
       </c>
       <c r="AV169" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="AW169" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="AX169" t="s">
         <v>250</v>
@@ -31901,12 +31910,12 @@
         <v>176</v>
       </c>
       <c r="BH169" t="s">
-        <v>250</v>
+        <v>192</v>
       </c>
     </row>
     <row r="170" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B170" t="s">
         <v>250</v>
@@ -32088,22 +32097,22 @@
     </row>
     <row r="171" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="C171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="D171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="E171" t="s">
         <v>176</v>
       </c>
       <c r="F171" t="s">
-        <v>217</v>
+        <v>176</v>
       </c>
       <c r="G171" t="s">
         <v>176</v>
@@ -32121,58 +32130,58 @@
         <v>176</v>
       </c>
       <c r="L171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="M171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="N171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="O171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="P171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="Q171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="R171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="S171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="T171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="U171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="V171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="W171" t="s">
-        <v>255</v>
+        <v>176</v>
       </c>
       <c r="X171" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="Y171" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="Z171" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="AA171" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="AB171" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="AC171" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="AD171" t="s">
         <v>176</v>
@@ -32196,7 +32205,7 @@
         <v>175</v>
       </c>
       <c r="AK171" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="AL171" t="s">
         <v>175</v>
@@ -32205,13 +32214,13 @@
         <v>175</v>
       </c>
       <c r="AN171" t="s">
-        <v>222</v>
+        <v>183</v>
       </c>
       <c r="AO171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="AP171" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="AQ171" t="s">
         <v>176</v>
@@ -32223,22 +32232,22 @@
         <v>176</v>
       </c>
       <c r="AT171" t="s">
-        <v>241</v>
+        <v>195</v>
       </c>
       <c r="AU171" t="s">
-        <v>276</v>
+        <v>176</v>
       </c>
       <c r="AV171" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="AW171" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="AX171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="AY171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="AZ171" t="s">
         <v>176</v>
@@ -32265,12 +32274,12 @@
         <v>176</v>
       </c>
       <c r="BH171" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
     </row>
     <row r="172" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B172" t="s">
         <v>192</v>
@@ -32444,7 +32453,7 @@
         <v>256</v>
       </c>
       <c r="BG172" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="BH172" t="s">
         <v>192</v>
@@ -32452,7 +32461,7 @@
     </row>
     <row r="173" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
-        <v>318</v>
+        <v>174</v>
       </c>
       <c r="B173" t="s">
         <v>192</v>
@@ -32626,7 +32635,7 @@
         <v>256</v>
       </c>
       <c r="BG173" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BH173" t="s">
         <v>192</v>
@@ -32634,7 +32643,7 @@
     </row>
     <row r="174" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B174" t="s">
         <v>192</v>
@@ -32808,7 +32817,7 @@
         <v>256</v>
       </c>
       <c r="BG174" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="BH174" t="s">
         <v>192</v>
@@ -32816,7 +32825,7 @@
     </row>
     <row r="175" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B175" t="s">
         <v>192</v>
@@ -32990,7 +32999,7 @@
         <v>256</v>
       </c>
       <c r="BG175" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="BH175" t="s">
         <v>192</v>
@@ -32998,7 +33007,7 @@
     </row>
     <row r="176" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B176" t="s">
         <v>192</v>
@@ -33172,9 +33181,191 @@
         <v>256</v>
       </c>
       <c r="BG176" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="BH176" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="177" spans="1:60" x14ac:dyDescent="0.3">
+      <c r="A177" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B177" t="s">
+        <v>192</v>
+      </c>
+      <c r="C177" t="s">
+        <v>192</v>
+      </c>
+      <c r="D177" t="s">
+        <v>192</v>
+      </c>
+      <c r="E177" t="s">
+        <v>176</v>
+      </c>
+      <c r="F177" t="s">
+        <v>217</v>
+      </c>
+      <c r="G177" t="s">
+        <v>176</v>
+      </c>
+      <c r="H177" t="s">
+        <v>176</v>
+      </c>
+      <c r="I177" t="s">
+        <v>176</v>
+      </c>
+      <c r="J177" t="s">
+        <v>176</v>
+      </c>
+      <c r="K177" t="s">
+        <v>176</v>
+      </c>
+      <c r="L177" t="s">
+        <v>192</v>
+      </c>
+      <c r="M177" t="s">
+        <v>192</v>
+      </c>
+      <c r="N177" t="s">
+        <v>192</v>
+      </c>
+      <c r="O177" t="s">
+        <v>192</v>
+      </c>
+      <c r="P177" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q177" t="s">
+        <v>192</v>
+      </c>
+      <c r="R177" t="s">
+        <v>192</v>
+      </c>
+      <c r="S177" t="s">
+        <v>192</v>
+      </c>
+      <c r="T177" t="s">
+        <v>192</v>
+      </c>
+      <c r="U177" t="s">
+        <v>192</v>
+      </c>
+      <c r="V177" t="s">
+        <v>192</v>
+      </c>
+      <c r="W177" t="s">
+        <v>255</v>
+      </c>
+      <c r="X177" t="s">
+        <v>192</v>
+      </c>
+      <c r="Y177" t="s">
+        <v>192</v>
+      </c>
+      <c r="Z177" t="s">
+        <v>192</v>
+      </c>
+      <c r="AA177" t="s">
+        <v>192</v>
+      </c>
+      <c r="AB177" t="s">
+        <v>192</v>
+      </c>
+      <c r="AC177" t="s">
+        <v>192</v>
+      </c>
+      <c r="AD177" t="s">
+        <v>176</v>
+      </c>
+      <c r="AE177" t="s">
+        <v>175</v>
+      </c>
+      <c r="AF177" t="s">
+        <v>175</v>
+      </c>
+      <c r="AG177" t="s">
+        <v>176</v>
+      </c>
+      <c r="AH177" t="s">
+        <v>250</v>
+      </c>
+      <c r="AI177" t="s">
+        <v>175</v>
+      </c>
+      <c r="AJ177" t="s">
+        <v>175</v>
+      </c>
+      <c r="AK177" t="s">
+        <v>192</v>
+      </c>
+      <c r="AL177" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM177" t="s">
+        <v>175</v>
+      </c>
+      <c r="AN177" t="s">
+        <v>222</v>
+      </c>
+      <c r="AO177" t="s">
+        <v>192</v>
+      </c>
+      <c r="AP177" t="s">
+        <v>182</v>
+      </c>
+      <c r="AQ177" t="s">
+        <v>176</v>
+      </c>
+      <c r="AR177" t="s">
+        <v>182</v>
+      </c>
+      <c r="AS177" t="s">
+        <v>176</v>
+      </c>
+      <c r="AT177" t="s">
+        <v>241</v>
+      </c>
+      <c r="AU177" t="s">
+        <v>276</v>
+      </c>
+      <c r="AV177" t="s">
+        <v>242</v>
+      </c>
+      <c r="AW177" t="s">
+        <v>242</v>
+      </c>
+      <c r="AX177" t="s">
+        <v>192</v>
+      </c>
+      <c r="AY177" t="s">
+        <v>192</v>
+      </c>
+      <c r="AZ177" t="s">
+        <v>176</v>
+      </c>
+      <c r="BA177" t="s">
+        <v>256</v>
+      </c>
+      <c r="BB177" t="s">
+        <v>256</v>
+      </c>
+      <c r="BC177" t="s">
+        <v>256</v>
+      </c>
+      <c r="BD177" t="s">
+        <v>256</v>
+      </c>
+      <c r="BE177" t="s">
+        <v>256</v>
+      </c>
+      <c r="BF177" t="s">
+        <v>256</v>
+      </c>
+      <c r="BG177" t="s">
+        <v>195</v>
+      </c>
+      <c r="BH177" t="s">
         <v>192</v>
       </c>
     </row>

</xml_diff>